<commit_message>
Add the skill recorder practice exercise
</commit_message>
<xml_diff>
--- a/skill-recorder-practice.xlsx
+++ b/skill-recorder-practice.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="1" r:id="Rc786c2d8df8448c4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Orders" sheetId="1" r:id="Rf8093ada8eb94a8d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -95,13 +95,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblOrders" displayName="tblOrders" ref="A4:E10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="5">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="tblOrders" displayName="tblOrders" ref="A4:F10" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A4:F10"/>
+  <x:tableColumns count="6">
     <x:tableColumn id="1" name="Order ID"/>
     <x:tableColumn id="2" name="Customer"/>
     <x:tableColumn id="3" name="Ordered"/>
     <x:tableColumn id="4" name="Shipped"/>
-    <x:tableColumn id="5" name="Context"/>
+    <x:tableColumn id="5" name="Cancelled"/>
+    <x:tableColumn id="6" name="Context"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -302,13 +304,14 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="13" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="13" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="11" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="11" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="48" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="13" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="50" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="43" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="47" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -342,7 +345,7 @@
       <x:c r="F3" s="2"/>
       <x:c r="G3" s="2"/>
     </x:row>
-    <x:row r="4" ht="30" customHeight="1">
+    <x:row r="4" ht="32" customHeight="1">
       <x:c r="A4" s="6" t="str">
         <x:v>Order ID</x:v>
       </x:c>
@@ -356,12 +359,14 @@
         <x:v>Shipped</x:v>
       </x:c>
       <x:c r="E4" s="6" t="str">
+        <x:v>Cancelled</x:v>
+      </x:c>
+      <x:c r="F4" s="6" t="str">
         <x:v>Context</x:v>
       </x:c>
-      <x:c r="F4" s="2"/>
       <x:c r="G4" s="2"/>
     </x:row>
-    <x:row r="5" ht="37" customHeight="1">
+    <x:row r="5" ht="38" customHeight="1">
       <x:c r="A5" s="2" t="str">
         <x:v>O-1001</x:v>
       </x:c>
@@ -374,13 +379,15 @@
       <x:c r="D5" s="7" t="n">
         <x:v>90</x:v>
       </x:c>
-      <x:c r="E5" s="8" t="str">
+      <x:c r="E5" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F5" s="8" t="str">
         <x:v>Replacement labels awaiting approval.</x:v>
       </x:c>
-      <x:c r="F5" s="2"/>
       <x:c r="G5" s="2"/>
     </x:row>
-    <x:row r="6" ht="37" customHeight="1">
+    <x:row r="6" ht="38" customHeight="1">
       <x:c r="A6" s="2" t="str">
         <x:v>O-1002</x:v>
       </x:c>
@@ -391,15 +398,17 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="D6" s="7" t="n">
-        <x:v>80</x:v>
-      </x:c>
-      <x:c r="E6" s="8" t="str">
-        <x:v>Complete.</x:v>
-      </x:c>
-      <x:c r="F6" s="2"/>
+        <x:v>70</x:v>
+      </x:c>
+      <x:c r="E6" s="7" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="F6" s="8" t="str">
+        <x:v>10 cancelled; balance shipped.</x:v>
+      </x:c>
       <x:c r="G6" s="2"/>
     </x:row>
-    <x:row r="7" ht="37" customHeight="1">
+    <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="2" t="str">
         <x:v>O-1003</x:v>
       </x:c>
@@ -412,13 +421,15 @@
       <x:c r="D7" s="7" t="n">
         <x:v>140</x:v>
       </x:c>
-      <x:c r="E7" s="8" t="str">
-        <x:v>Customer requested split delivery.</x:v>
-      </x:c>
-      <x:c r="F7" s="2"/>
+      <x:c r="E7" s="7" t="n">
+        <x:v>20</x:v>
+      </x:c>
+      <x:c r="F7" s="8" t="str">
+        <x:v>20 cancelled; split delivery agreed.</x:v>
+      </x:c>
       <x:c r="G7" s="2"/>
     </x:row>
-    <x:row r="8" ht="37" customHeight="1">
+    <x:row r="8" ht="38" customHeight="1">
       <x:c r="A8" s="2" t="str">
         <x:v>O-1004</x:v>
       </x:c>
@@ -431,11 +442,13 @@
       <x:c r="D8" s="7" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E8" s="8" t="str"/>
-      <x:c r="F8" s="2"/>
+      <x:c r="E8" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F8" s="8" t="str"/>
       <x:c r="G8" s="2"/>
     </x:row>
-    <x:row r="9" ht="37" customHeight="1">
+    <x:row r="9" ht="38" customHeight="1">
       <x:c r="A9" s="2" t="str">
         <x:v>O-1005</x:v>
       </x:c>
@@ -448,13 +461,15 @@
       <x:c r="D9" s="7" t="n">
         <x:v>125</x:v>
       </x:c>
-      <x:c r="E9" s="8" t="str">
-        <x:v>Carrier pickup moved to Friday.</x:v>
-      </x:c>
-      <x:c r="F9" s="2"/>
+      <x:c r="E9" s="7" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="F9" s="8" t="str">
+        <x:v>5 cancelled; Friday pickup planned.</x:v>
+      </x:c>
       <x:c r="G9" s="2"/>
     </x:row>
-    <x:row r="10" ht="37" customHeight="1">
+    <x:row r="10" ht="38" customHeight="1">
       <x:c r="A10" s="2" t="str">
         <x:v>O-1006</x:v>
       </x:c>
@@ -467,10 +482,12 @@
       <x:c r="D10" s="7" t="n">
         <x:v>100</x:v>
       </x:c>
-      <x:c r="E10" s="8" t="str">
+      <x:c r="E10" s="7" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F10" s="8" t="str">
         <x:v>Complete.</x:v>
       </x:c>
-      <x:c r="F10" s="2"/>
       <x:c r="G10" s="2"/>
     </x:row>
     <x:row r="11">
@@ -530,7 +547,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2c49d46ee55c4b8b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1fedb13134344c94"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>